<commit_message>
mejora interfaz de consulta y listado de habitaciones
</commit_message>
<xml_diff>
--- a/Documentacion/Pruebas/Pruebas_Funcionales_Hotel_Pacific_Reef.xlsx
+++ b/Documentacion/Pruebas/Pruebas_Funcionales_Hotel_Pacific_Reef.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blank\Desktop\Ing de software\Hotel-Pacific-Reef\Documentacion\Pruebas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FE89DB55-B7E4-4987-BC26-1CD6C5FFD4B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D548814-C80F-4BDE-82F7-3D2B8E4986A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10755" yWindow="825" windowWidth="15555" windowHeight="11295" xr2:uid="{D7AA81E4-BD21-49A3-BCC0-B9C86846883E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D7AA81E4-BD21-49A3-BCC0-B9C86846883E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -59,9 +59,6 @@
     <t xml:space="preserve">Resultado Obtenido </t>
   </si>
   <si>
-    <t>Estado</t>
-  </si>
-  <si>
     <t>CP-01</t>
   </si>
   <si>
@@ -96,6 +93,9 @@
   </si>
   <si>
     <t xml:space="preserve">Aprobado </t>
+  </si>
+  <si>
+    <t>aprobado</t>
   </si>
 </sst>
 </file>
@@ -480,7 +480,7 @@
     <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -500,53 +500,53 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="135" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" t="s">
         <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
integra servicio de clima y amplia pruebas funcionales
</commit_message>
<xml_diff>
--- a/Documentacion/Pruebas/Pruebas_Funcionales_Hotel_Pacific_Reef.xlsx
+++ b/Documentacion/Pruebas/Pruebas_Funcionales_Hotel_Pacific_Reef.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\blank\Desktop\Ing de software\Hotel-Pacific-Reef\Documentacion\Pruebas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D548814-C80F-4BDE-82F7-3D2B8E4986A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6366D4-DFFD-4610-929A-323EE537C6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D7AA81E4-BD21-49A3-BCC0-B9C86846883E}"/>
+    <workbookView xWindow="-450" yWindow="0" windowWidth="17175" windowHeight="15585" xr2:uid="{D7AA81E4-BD21-49A3-BCC0-B9C86846883E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
   <si>
     <t>Historia de ususario</t>
   </si>
@@ -95,7 +95,88 @@
     <t xml:space="preserve">Aprobado </t>
   </si>
   <si>
-    <t>aprobado</t>
+    <t xml:space="preserve">Estado </t>
+  </si>
+  <si>
+    <t>CP-03</t>
+  </si>
+  <si>
+    <t>HU-04</t>
+  </si>
+  <si>
+    <t>Validacion de fecha de entrada</t>
+  </si>
+  <si>
+    <t>Intentar seleccionar una fecha anterior a la fecha actual</t>
+  </si>
+  <si>
+    <t>El sistema debe impedir seleccionar fechas de entrada anteriores a la fecha actual</t>
+  </si>
+  <si>
+    <t>El calendario bloquea las fechas anteriores a la fecha actual y no permite seleccionarlas</t>
+  </si>
+  <si>
+    <t>CP-04</t>
+  </si>
+  <si>
+    <t>Validacion de fechas de reserva</t>
+  </si>
+  <si>
+    <t>Entrada: 10/10/2026        Salida: 09/10/2026</t>
+  </si>
+  <si>
+    <t>El sistema debe rechazar la reserva si la fecha de salida es anterior o igual a la fecha de entrada</t>
+  </si>
+  <si>
+    <t>El sistema rechaza la solicitud y muestra el mensaje "La fecha de salida debe ser porterior a al fecha de entrada"</t>
+  </si>
+  <si>
+    <t>CP-05</t>
+  </si>
+  <si>
+    <t>Validacion de disponibilidad al reservar</t>
+  </si>
+  <si>
+    <t>El sistema debe impedir registrar una reserva que se superponga con una reserva confirmada</t>
+  </si>
+  <si>
+    <t>El sistema rechaza la solicitud y muestra el mensaje "La habitacion no esta disponible para las fechas seleccionadas"</t>
+  </si>
+  <si>
+    <t>Habitacion 101-   Entrada: 11/10/2026        Salida: 12/10/2026</t>
+  </si>
+  <si>
+    <t>CP-06</t>
+  </si>
+  <si>
+    <t>Registro de reserva</t>
+  </si>
+  <si>
+    <t>Habitacion 101-   Entrada: 10/10/2026        Salida: 13/10/2026</t>
+  </si>
+  <si>
+    <t>Registrar una reserva confirmada de 3 noches y almacenarla en la base de datos</t>
+  </si>
+  <si>
+    <t>Se registra correctamente la Reserva #2 para la habitacion 101 por 3 noches y queda almacenada con estado confirmada</t>
+  </si>
+  <si>
+    <t>CP-07</t>
+  </si>
+  <si>
+    <t>HU-05</t>
+  </si>
+  <si>
+    <t>Cálculo del monto de reserva (30%)</t>
+  </si>
+  <si>
+    <t>Habitacion 101 - 3 noches - Precio por noche: $45.000</t>
+  </si>
+  <si>
+    <t>Calcular total de estadía en $135.000 y monto de reserva del 30% en $40.500</t>
+  </si>
+  <si>
+    <t>El sistema calcula 3 noches, total $135.000 y monto de reserva $40.500</t>
   </si>
 </sst>
 </file>
@@ -131,10 +212,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -470,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEE1D065-B04C-4626-9BD4-A496AA0A57C5}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.42578125" customWidth="1"/>
@@ -549,6 +633,121 @@
         <v>17</v>
       </c>
     </row>
+    <row r="4" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>